<commit_message>
fix: give every applicant type the 000 document set
</commit_message>
<xml_diff>
--- a/mosip_master/xlsx/applicant_valid_document.xlsx
+++ b/mosip_master/xlsx/applicant_valid_document.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="955" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="890" uniqueCount="41">
   <si>
     <t>lang_code</t>
   </si>
@@ -506,7 +506,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E191"/>
+  <dimension ref="A1:E178"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
@@ -738,7 +738,7 @@
         <v>22</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>12</v>
@@ -755,10 +755,10 @@
         <v>22</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>9</v>
@@ -775,7 +775,7 @@
         <v>14</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>9</v>
@@ -792,7 +792,7 @@
         <v>14</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>9</v>
@@ -806,10 +806,10 @@
         <v>22</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>9</v>
@@ -823,10 +823,10 @@
         <v>22</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>9</v>
@@ -854,13 +854,13 @@
         <v>5</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>9</v>
@@ -871,13 +871,13 @@
         <v>5</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>9</v>
@@ -894,7 +894,7 @@
         <v>7</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>9</v>
@@ -908,10 +908,10 @@
         <v>23</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>9</v>
@@ -925,10 +925,10 @@
         <v>23</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>9</v>
@@ -942,10 +942,10 @@
         <v>23</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>9</v>
@@ -959,10 +959,10 @@
         <v>23</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>9</v>
@@ -976,10 +976,10 @@
         <v>23</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>9</v>
@@ -993,10 +993,10 @@
         <v>23</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>9</v>
@@ -1010,10 +1010,10 @@
         <v>23</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>9</v>
@@ -1024,13 +1024,13 @@
         <v>5</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>9</v>
@@ -1041,13 +1041,13 @@
         <v>5</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>40</v>
+        <v>7</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>9</v>
@@ -1064,7 +1064,7 @@
         <v>7</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>9</v>
@@ -1078,10 +1078,10 @@
         <v>24</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>9</v>
@@ -1095,10 +1095,10 @@
         <v>24</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>9</v>
@@ -1112,10 +1112,10 @@
         <v>24</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>9</v>
@@ -1129,10 +1129,10 @@
         <v>24</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>9</v>
@@ -1146,10 +1146,10 @@
         <v>24</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>9</v>
@@ -1163,10 +1163,10 @@
         <v>24</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>9</v>
@@ -1180,10 +1180,10 @@
         <v>24</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>9</v>
@@ -1194,13 +1194,13 @@
         <v>5</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>9</v>
@@ -1211,13 +1211,13 @@
         <v>5</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>40</v>
+        <v>7</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>9</v>
@@ -1228,13 +1228,13 @@
         <v>5</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E43" s="2" t="s">
         <v>9</v>
@@ -1245,13 +1245,13 @@
         <v>5</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>9</v>
@@ -1265,10 +1265,10 @@
         <v>25</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>9</v>
@@ -1282,10 +1282,10 @@
         <v>25</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E46" s="2" t="s">
         <v>9</v>
@@ -1299,10 +1299,10 @@
         <v>25</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="E47" s="2" t="s">
         <v>9</v>
@@ -1316,7 +1316,7 @@
         <v>25</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>12</v>
@@ -1333,10 +1333,10 @@
         <v>25</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="E49" s="2" t="s">
         <v>9</v>
@@ -1350,10 +1350,10 @@
         <v>25</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E50" s="2" t="s">
         <v>9</v>
@@ -1364,13 +1364,13 @@
         <v>5</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E51" s="2" t="s">
         <v>9</v>
@@ -1381,13 +1381,13 @@
         <v>5</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="E52" s="2" t="s">
         <v>9</v>
@@ -1398,13 +1398,13 @@
         <v>5</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C53" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="E53" s="2" t="s">
         <v>9</v>
@@ -1415,13 +1415,13 @@
         <v>5</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>40</v>
+        <v>13</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>9</v>
@@ -1435,10 +1435,10 @@
         <v>26</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>9</v>
@@ -1452,10 +1452,10 @@
         <v>26</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E56" s="2" t="s">
         <v>9</v>
@@ -1469,10 +1469,10 @@
         <v>26</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>9</v>
@@ -1486,7 +1486,7 @@
         <v>26</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="D58" s="2" t="s">
         <v>12</v>
@@ -1503,10 +1503,10 @@
         <v>26</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="E59" s="2" t="s">
         <v>9</v>
@@ -1520,10 +1520,10 @@
         <v>26</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E60" s="2" t="s">
         <v>9</v>
@@ -1534,13 +1534,13 @@
         <v>5</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E61" s="2" t="s">
         <v>9</v>
@@ -1551,13 +1551,13 @@
         <v>5</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="E62" s="2" t="s">
         <v>9</v>
@@ -1568,13 +1568,13 @@
         <v>5</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E63" s="2" t="s">
         <v>9</v>
@@ -1585,13 +1585,13 @@
         <v>5</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="E64" s="2" t="s">
         <v>9</v>
@@ -1605,10 +1605,10 @@
         <v>27</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="E65" s="2" t="s">
         <v>9</v>
@@ -1622,10 +1622,10 @@
         <v>27</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E66" s="2" t="s">
         <v>9</v>
@@ -1639,10 +1639,10 @@
         <v>27</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="E67" s="2" t="s">
         <v>9</v>
@@ -1656,7 +1656,7 @@
         <v>27</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D68" s="2" t="s">
         <v>12</v>
@@ -1673,10 +1673,10 @@
         <v>27</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="E69" s="2" t="s">
         <v>9</v>
@@ -1690,10 +1690,10 @@
         <v>27</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E70" s="2" t="s">
         <v>9</v>
@@ -1704,13 +1704,13 @@
         <v>5</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="E71" s="2" t="s">
         <v>9</v>
@@ -1721,13 +1721,13 @@
         <v>5</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C72" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="E72" s="2" t="s">
         <v>9</v>
@@ -1738,13 +1738,13 @@
         <v>5</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>40</v>
+        <v>7</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="E73" s="2" t="s">
         <v>9</v>
@@ -1758,10 +1758,10 @@
         <v>28</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E74" s="2" t="s">
         <v>9</v>
@@ -1775,10 +1775,10 @@
         <v>28</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E75" s="2" t="s">
         <v>9</v>
@@ -1792,10 +1792,10 @@
         <v>28</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E76" s="2" t="s">
         <v>9</v>
@@ -1809,10 +1809,10 @@
         <v>28</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="E77" s="2" t="s">
         <v>9</v>
@@ -1826,7 +1826,7 @@
         <v>28</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D78" s="2" t="s">
         <v>12</v>
@@ -1843,10 +1843,10 @@
         <v>28</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="E79" s="2" t="s">
         <v>9</v>
@@ -1860,10 +1860,10 @@
         <v>28</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E80" s="2" t="s">
         <v>9</v>
@@ -1874,13 +1874,13 @@
         <v>5</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="E81" s="2" t="s">
         <v>9</v>
@@ -1891,13 +1891,13 @@
         <v>5</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C82" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="E82" s="2" t="s">
         <v>9</v>
@@ -1908,13 +1908,13 @@
         <v>5</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>40</v>
+        <v>7</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="E83" s="2" t="s">
         <v>9</v>
@@ -1925,10 +1925,10 @@
         <v>5</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="D84" s="2" t="s">
         <v>12</v>
@@ -1942,13 +1942,13 @@
         <v>5</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E85" s="2" t="s">
         <v>9</v>
@@ -1962,10 +1962,10 @@
         <v>29</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E86" s="2" t="s">
         <v>9</v>
@@ -1979,10 +1979,10 @@
         <v>29</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="E87" s="2" t="s">
         <v>9</v>
@@ -1996,10 +1996,10 @@
         <v>29</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E88" s="2" t="s">
         <v>9</v>
@@ -2013,10 +2013,10 @@
         <v>29</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="E89" s="2" t="s">
         <v>9</v>
@@ -2030,10 +2030,10 @@
         <v>29</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="E90" s="2" t="s">
         <v>9</v>
@@ -2044,13 +2044,13 @@
         <v>5</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="E91" s="2" t="s">
         <v>9</v>
@@ -2061,13 +2061,13 @@
         <v>5</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="E92" s="2" t="s">
         <v>9</v>
@@ -2078,13 +2078,13 @@
         <v>5</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="E93" s="2" t="s">
         <v>9</v>
@@ -2095,13 +2095,13 @@
         <v>5</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="E94" s="2" t="s">
         <v>9</v>
@@ -2112,13 +2112,13 @@
         <v>5</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E95" s="2" t="s">
         <v>9</v>
@@ -2132,10 +2132,10 @@
         <v>30</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E96" s="2" t="s">
         <v>9</v>
@@ -2149,10 +2149,10 @@
         <v>30</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="E97" s="2" t="s">
         <v>9</v>
@@ -2166,10 +2166,10 @@
         <v>30</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E98" s="2" t="s">
         <v>9</v>
@@ -2183,10 +2183,10 @@
         <v>30</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="E99" s="2" t="s">
         <v>9</v>
@@ -2200,10 +2200,10 @@
         <v>30</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="E100" s="2" t="s">
         <v>9</v>
@@ -2217,10 +2217,10 @@
         <v>30</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E101" s="2" t="s">
         <v>9</v>
@@ -2231,13 +2231,13 @@
         <v>5</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E102" s="2" t="s">
         <v>9</v>
@@ -2248,13 +2248,13 @@
         <v>5</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="D103" s="2" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="E103" s="2" t="s">
         <v>9</v>
@@ -2265,13 +2265,13 @@
         <v>5</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C104" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="E104" s="2" t="s">
         <v>9</v>
@@ -2282,13 +2282,13 @@
         <v>5</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>40</v>
+        <v>13</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="E105" s="2" t="s">
         <v>9</v>
@@ -2299,13 +2299,13 @@
         <v>5</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E106" s="2" t="s">
         <v>9</v>
@@ -2316,13 +2316,13 @@
         <v>5</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="D107" s="2" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="E107" s="2" t="s">
         <v>9</v>
@@ -2333,13 +2333,13 @@
         <v>5</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="E108" s="2" t="s">
         <v>9</v>
@@ -2353,10 +2353,10 @@
         <v>33</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E109" s="2" t="s">
         <v>9</v>
@@ -2370,10 +2370,10 @@
         <v>33</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E110" s="2" t="s">
         <v>9</v>
@@ -2387,10 +2387,10 @@
         <v>33</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="D111" s="2" t="s">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="E111" s="2" t="s">
         <v>9</v>
@@ -2404,10 +2404,10 @@
         <v>33</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>7</v>
+        <v>40</v>
       </c>
       <c r="D112" s="2" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="E112" s="2" t="s">
         <v>9</v>
@@ -2418,13 +2418,13 @@
         <v>5</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E113" s="2" t="s">
         <v>9</v>
@@ -2435,13 +2435,13 @@
         <v>5</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E114" s="2" t="s">
         <v>9</v>
@@ -2452,13 +2452,13 @@
         <v>5</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="E115" s="2" t="s">
         <v>9</v>
@@ -2469,13 +2469,13 @@
         <v>5</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E116" s="2" t="s">
         <v>9</v>
@@ -2486,13 +2486,13 @@
         <v>5</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D117" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E117" s="2" t="s">
         <v>9</v>
@@ -2503,13 +2503,13 @@
         <v>5</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E118" s="2" t="s">
         <v>9</v>
@@ -2520,13 +2520,13 @@
         <v>5</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="D119" s="2" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="E119" s="2" t="s">
         <v>9</v>
@@ -2540,10 +2540,10 @@
         <v>34</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E120" s="2" t="s">
         <v>9</v>
@@ -2557,10 +2557,10 @@
         <v>34</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="D121" s="2" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E121" s="2" t="s">
         <v>9</v>
@@ -2574,10 +2574,10 @@
         <v>34</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="E122" s="2" t="s">
         <v>9</v>
@@ -2591,10 +2591,10 @@
         <v>34</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>7</v>
+        <v>40</v>
       </c>
       <c r="D123" s="2" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="E123" s="2" t="s">
         <v>9</v>
@@ -2605,13 +2605,13 @@
         <v>5</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D124" s="2" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E124" s="2" t="s">
         <v>9</v>
@@ -2622,13 +2622,13 @@
         <v>5</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="D125" s="2" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E125" s="2" t="s">
         <v>9</v>
@@ -2639,13 +2639,13 @@
         <v>5</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="D126" s="2" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="E126" s="2" t="s">
         <v>9</v>
@@ -2656,13 +2656,13 @@
         <v>5</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D127" s="2" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E127" s="2" t="s">
         <v>9</v>
@@ -2673,13 +2673,13 @@
         <v>5</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D128" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E128" s="2" t="s">
         <v>9</v>
@@ -2690,13 +2690,13 @@
         <v>5</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="D129" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E129" s="2" t="s">
         <v>9</v>
@@ -2707,13 +2707,13 @@
         <v>5</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="E130" s="2" t="s">
         <v>9</v>
@@ -2724,13 +2724,13 @@
         <v>5</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C131" s="2" t="s">
         <v>20</v>
       </c>
       <c r="D131" s="2" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="E131" s="2" t="s">
         <v>9</v>
@@ -2741,13 +2741,13 @@
         <v>5</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="D132" s="2" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="E132" s="2" t="s">
         <v>9</v>
@@ -2761,10 +2761,10 @@
         <v>35</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="D133" s="2" t="s">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="E133" s="2" t="s">
         <v>9</v>
@@ -2778,10 +2778,10 @@
         <v>35</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>7</v>
+        <v>40</v>
       </c>
       <c r="D134" s="2" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="E134" s="2" t="s">
         <v>9</v>
@@ -2792,13 +2792,13 @@
         <v>5</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C135" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D135" s="2" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E135" s="2" t="s">
         <v>9</v>
@@ -2809,13 +2809,13 @@
         <v>5</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C136" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D136" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E136" s="2" t="s">
         <v>9</v>
@@ -2826,13 +2826,13 @@
         <v>5</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D137" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E137" s="2" t="s">
         <v>9</v>
@@ -2843,13 +2843,13 @@
         <v>5</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D138" s="2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E138" s="2" t="s">
         <v>9</v>
@@ -2860,13 +2860,13 @@
         <v>5</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C139" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D139" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E139" s="2" t="s">
         <v>9</v>
@@ -2877,13 +2877,13 @@
         <v>5</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C140" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D140" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E140" s="2" t="s">
         <v>9</v>
@@ -2894,13 +2894,13 @@
         <v>5</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D141" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E141" s="2" t="s">
         <v>9</v>
@@ -2911,13 +2911,13 @@
         <v>5</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="D142" s="2" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="E142" s="2" t="s">
         <v>9</v>
@@ -2928,13 +2928,13 @@
         <v>5</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="D143" s="2" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="E143" s="2" t="s">
         <v>9</v>
@@ -2948,10 +2948,10 @@
         <v>36</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="D144" s="2" t="s">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="E144" s="2" t="s">
         <v>9</v>
@@ -2965,10 +2965,10 @@
         <v>36</v>
       </c>
       <c r="C145" s="2" t="s">
-        <v>7</v>
+        <v>40</v>
       </c>
       <c r="D145" s="2" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="E145" s="2" t="s">
         <v>9</v>
@@ -2979,13 +2979,13 @@
         <v>5</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C146" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D146" s="2" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E146" s="2" t="s">
         <v>9</v>
@@ -2996,13 +2996,13 @@
         <v>5</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C147" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D147" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E147" s="2" t="s">
         <v>9</v>
@@ -3013,13 +3013,13 @@
         <v>5</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D148" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E148" s="2" t="s">
         <v>9</v>
@@ -3030,13 +3030,13 @@
         <v>5</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D149" s="2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E149" s="2" t="s">
         <v>9</v>
@@ -3047,13 +3047,13 @@
         <v>5</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C150" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D150" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E150" s="2" t="s">
         <v>9</v>
@@ -3064,13 +3064,13 @@
         <v>5</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C151" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D151" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E151" s="2" t="s">
         <v>9</v>
@@ -3081,13 +3081,13 @@
         <v>5</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C152" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D152" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E152" s="2" t="s">
         <v>9</v>
@@ -3098,13 +3098,13 @@
         <v>5</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="D153" s="2" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="E153" s="2" t="s">
         <v>9</v>
@@ -3115,13 +3115,13 @@
         <v>5</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C154" s="2" t="s">
         <v>20</v>
       </c>
       <c r="D154" s="2" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="E154" s="2" t="s">
         <v>9</v>
@@ -3132,13 +3132,13 @@
         <v>5</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="D155" s="2" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="E155" s="2" t="s">
         <v>9</v>
@@ -3149,13 +3149,13 @@
         <v>5</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="D156" s="2" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="E156" s="2" t="s">
         <v>9</v>
@@ -3166,7 +3166,7 @@
         <v>5</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C157" s="2" t="s">
         <v>7</v>
@@ -3183,7 +3183,7 @@
         <v>5</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C158" s="2" t="s">
         <v>7</v>
@@ -3200,7 +3200,7 @@
         <v>5</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C159" s="2" t="s">
         <v>7</v>
@@ -3217,10 +3217,10 @@
         <v>5</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="D160" s="2" t="s">
         <v>12</v>
@@ -3234,13 +3234,13 @@
         <v>5</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C161" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D161" s="2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E161" s="2" t="s">
         <v>9</v>
@@ -3251,13 +3251,13 @@
         <v>5</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C162" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D162" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E162" s="2" t="s">
         <v>9</v>
@@ -3268,13 +3268,13 @@
         <v>5</v>
       </c>
       <c r="B163" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C163" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D163" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E163" s="2" t="s">
         <v>9</v>
@@ -3285,13 +3285,13 @@
         <v>5</v>
       </c>
       <c r="B164" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C164" s="2" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="D164" s="2" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E164" s="2" t="s">
         <v>9</v>
@@ -3302,13 +3302,13 @@
         <v>5</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C165" s="2" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="D165" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E165" s="2" t="s">
         <v>9</v>
@@ -3319,13 +3319,13 @@
         <v>5</v>
       </c>
       <c r="B166" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C166" s="2" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="D166" s="2" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="E166" s="2" t="s">
         <v>9</v>
@@ -3336,13 +3336,13 @@
         <v>5</v>
       </c>
       <c r="B167" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C167" s="2" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="D167" s="2" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="E167" s="2" t="s">
         <v>9</v>
@@ -3353,7 +3353,7 @@
         <v>5</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C168" s="2" t="s">
         <v>7</v>
@@ -3370,7 +3370,7 @@
         <v>5</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C169" s="2" t="s">
         <v>7</v>
@@ -3387,7 +3387,7 @@
         <v>5</v>
       </c>
       <c r="B170" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C170" s="2" t="s">
         <v>7</v>
@@ -3404,10 +3404,10 @@
         <v>5</v>
       </c>
       <c r="B171" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="D171" s="2" t="s">
         <v>12</v>
@@ -3421,13 +3421,13 @@
         <v>5</v>
       </c>
       <c r="B172" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C172" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D172" s="2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E172" s="2" t="s">
         <v>9</v>
@@ -3438,13 +3438,13 @@
         <v>5</v>
       </c>
       <c r="B173" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C173" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D173" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E173" s="2" t="s">
         <v>9</v>
@@ -3455,13 +3455,13 @@
         <v>5</v>
       </c>
       <c r="B174" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C174" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D174" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E174" s="2" t="s">
         <v>9</v>
@@ -3472,13 +3472,13 @@
         <v>5</v>
       </c>
       <c r="B175" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C175" s="2" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="D175" s="2" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E175" s="2" t="s">
         <v>9</v>
@@ -3489,13 +3489,13 @@
         <v>5</v>
       </c>
       <c r="B176" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C176" s="2" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="D176" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E176" s="2" t="s">
         <v>9</v>
@@ -3506,13 +3506,13 @@
         <v>5</v>
       </c>
       <c r="B177" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C177" s="2" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="D177" s="2" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="E177" s="2" t="s">
         <v>9</v>
@@ -3523,236 +3523,15 @@
         <v>5</v>
       </c>
       <c r="B178" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C178" s="2" t="s">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="D178" s="2" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="E178" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A179" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B179" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C179" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D179" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E179" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A180" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B180" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C180" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D180" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="E180" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A181" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B181" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C181" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D181" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E181" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A182" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B182" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C182" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D182" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E182" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A183" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B183" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C183" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D183" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E183" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A184" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B184" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C184" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D184" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E184" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A185" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B185" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C185" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D185" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E185" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A186" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B186" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C186" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D186" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E186" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A187" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B187" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C187" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D187" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E187" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A188" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B188" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C188" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D188" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E188" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A189" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B189" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C189" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D189" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E189" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A190" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B190" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C190" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D190" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E190" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A191" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B191" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C191" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D191" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="E191" s="2" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: offer birth certificate as identity proof for child applicant types
</commit_message>
<xml_diff>
--- a/mosip_master/xlsx/applicant_valid_document.xlsx
+++ b/mosip_master/xlsx/applicant_valid_document.xlsx
@@ -690,7 +690,7 @@
         <v>7</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>9</v>
@@ -707,7 +707,7 @@
         <v>7</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>9</v>
@@ -724,7 +724,7 @@
         <v>7</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>9</v>
@@ -1030,7 +1030,7 @@
         <v>7</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>9</v>
@@ -1047,7 +1047,7 @@
         <v>7</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>9</v>
@@ -1064,7 +1064,7 @@
         <v>7</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>9</v>
@@ -1370,7 +1370,7 @@
         <v>7</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E51" s="2" t="s">
         <v>9</v>
@@ -1387,7 +1387,7 @@
         <v>7</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E52" s="2" t="s">
         <v>9</v>
@@ -1404,7 +1404,7 @@
         <v>7</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E53" s="2" t="s">
         <v>9</v>
@@ -1710,7 +1710,7 @@
         <v>7</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E71" s="2" t="s">
         <v>9</v>
@@ -1727,7 +1727,7 @@
         <v>7</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E72" s="2" t="s">
         <v>9</v>
@@ -1744,7 +1744,7 @@
         <v>7</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E73" s="2" t="s">
         <v>9</v>
@@ -2050,7 +2050,7 @@
         <v>7</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E91" s="2" t="s">
         <v>9</v>
@@ -2067,7 +2067,7 @@
         <v>7</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E92" s="2" t="s">
         <v>9</v>
@@ -2084,7 +2084,7 @@
         <v>7</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E93" s="2" t="s">
         <v>9</v>
@@ -2424,7 +2424,7 @@
         <v>7</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E113" s="2" t="s">
         <v>9</v>
@@ -2441,7 +2441,7 @@
         <v>7</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E114" s="2" t="s">
         <v>9</v>
@@ -2458,7 +2458,7 @@
         <v>7</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E115" s="2" t="s">
         <v>9</v>
@@ -2798,7 +2798,7 @@
         <v>7</v>
       </c>
       <c r="D135" s="2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E135" s="2" t="s">
         <v>9</v>
@@ -2815,7 +2815,7 @@
         <v>7</v>
       </c>
       <c r="D136" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E136" s="2" t="s">
         <v>9</v>
@@ -2832,7 +2832,7 @@
         <v>7</v>
       </c>
       <c r="D137" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E137" s="2" t="s">
         <v>9</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="D157" s="2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E157" s="2" t="s">
         <v>9</v>
@@ -3189,7 +3189,7 @@
         <v>7</v>
       </c>
       <c r="D158" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E158" s="2" t="s">
         <v>9</v>
@@ -3206,7 +3206,7 @@
         <v>7</v>
       </c>
       <c r="D159" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E159" s="2" t="s">
         <v>9</v>

</xml_diff>